<commit_message>
CUS-X01: DMS-XML velformethed + XSD-strukturvalidering (advisory) — katalog v0.2.0, suite+tests, CI markeret Daekket, regenereret pakke
</commit_message>
<xml_diff>
--- a/docs/Customs-Analytics_Regel-sporbarhedsmatrix.xlsx
+++ b/docs/Customs-Analytics_Regel-sporbarhedsmatrix.xlsx
@@ -479,7 +479,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>0.1.0</t>
+          <t>0.2.0</t>
         </is>
       </c>
     </row>
@@ -491,7 +491,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-07-01</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -711,32 +711,32 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>XSD-strukturvalidering mod H1/I1-skema</t>
+          <t>DMS-XML velformethed + strukturvalidering mod H1/I1-skema</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Rød — handling krævet</t>
+          <t>Gul — gennemse</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Planlagt (udkast)</t>
+          <t>Implementeret</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Toldstyrelsen skat/dms-public — H1/I1 XSD-skemaer (reference/xsds/).</t>
+          <t>Toldstyrelsen skat/dms-public — H1 V2.5 / I1 V2.3 XSD-skemaer (reference/xsds/).</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>(ikke wired — XSD'er foreligger i reference/xsds/)</t>
+          <t>customs/xsd_validation.py:validate_dms_xml</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>(planlagt)</t>
+          <t>tests/test_xsd_validation.py; validation/scenarios.py (CUS-X01)</t>
         </is>
       </c>
     </row>

</xml_diff>